<commit_message>
Revert "Merge branch 'm-matsumoto' into saito-comment"
This reverts commit 0259a82b5b0d9bb5109f220beab4f117ae2a2876, reversing
changes made to 5cbcc3035065f0d66f21d9377fa9a0e80a3b8eab.
</commit_message>
<xml_diff>
--- a/paiza-training/02_スキルチェック一覧.xlsx
+++ b/paiza-training/02_スキルチェック一覧.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\CSV2404-0002\backup\m-matsumoto\入社教育\2. C#基礎\Paiza-Training\paiza-training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B71E9E-FB7B-4ECE-911A-27CA0DF166EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB0DE56-9D4E-4713-8FD4-34BD801E517D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="45">
   <si>
     <t>日付</t>
   </si>
@@ -322,30 +322,6 @@
   </si>
   <si>
     <t xml:space="preserve"> 79分14秒</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>solution_4.cs</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>solution_5.cs</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>123分57秒</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>A078</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>93分29秒</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>B155</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -1107,123 +1083,66 @@
       <c r="A18" s="10">
         <v>15</v>
       </c>
-      <c r="B18" s="6">
-        <v>45876</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F18" s="1">
-        <v>100</v>
-      </c>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
       <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="10">
         <v>16</v>
       </c>
-      <c r="B19" s="6">
-        <v>45876</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F19" s="1">
-        <v>100</v>
-      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
       <c r="G19" s="1"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="10">
         <v>17</v>
       </c>
-      <c r="B20" s="6">
-        <v>45876</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>37</v>
-      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="10">
         <v>18</v>
       </c>
-      <c r="B21" s="6">
-        <v>45876</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F21" s="1">
-        <v>80</v>
-      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="10">
         <v>19</v>
       </c>
-      <c r="B22" s="6">
-        <v>45876</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F22" s="1">
-        <v>100</v>
-      </c>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
       <c r="G22" s="1"/>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="10">
         <v>20</v>
       </c>
-      <c r="B23" s="6">
-        <v>45876</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F23" s="1">
-        <v>0</v>
-      </c>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
       <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7">

</xml_diff>